<commit_message>
Add word "regnskab" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -497,9 +497,80 @@
         <v>Lapses</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>dc7a4e55-65f9-4b44-84c6-4fe4c7ae5838</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="C2" t="str">
+        <v>regnskab</v>
+      </c>
+      <c r="D2" t="str">
+        <v>regnskab</v>
+      </c>
+      <c r="E2" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F2" t="str">
+        <v>et</v>
+      </c>
+      <c r="G2" t="str">
+        <v>-et, -er, -erne</v>
+      </c>
+      <c r="H2" t="str">
+        <v>[ˈʁɑjnˌsgæˀb]</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://static.ordnet.dk/mp3/11042/11042574_1.mp3</v>
+      </c>
+      <c r="J2" t="str">
+        <v>opgørelse over indtægter og udgifter der viser resultatet i en bestemt periode for en økonomisk aktivitet, fx et firmas eller en forretnings drift eller et bestemt projekt</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Accounting</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Få besked når Solbjerggaard afleverer regnskab, flytter eller lukker.</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Solbjerggaard i Nordborg - CVR API</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://cvrapi.dk/virksomhed/dk/paul-bonde-christiansen/31813131</v>
+      </c>
+      <c r="O2" t="str">
+        <v>https://cvrapi.dk/virksomhed/dk/paul-bonde-christiansen/31813131#:~:text=regnskab</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -508,23 +579,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -591,8 +662,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="28.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "ankommet" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -399,36 +399,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AB4"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -674,9 +674,95 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>c1ebb2ab-a57e-4cca-8b06-bf5e494f9419</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-07-22</v>
+      </c>
+      <c r="C4" t="str">
+        <v>ankommet</v>
+      </c>
+      <c r="D4" t="str">
+        <v>ankomme</v>
+      </c>
+      <c r="E4" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>-r, ankom, -t</v>
+      </c>
+      <c r="H4" t="str">
+        <v>[ˈanˌkʌmˀə]</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://static.ordnet.dk/mp3/11001/11001850_1.mp3</v>
+      </c>
+      <c r="J4" t="str">
+        <v>komme til et bestemt sted efter at have tilbagelagt en vis afstand om person eller transportmiddel</v>
+      </c>
+      <c r="K4" t="str">
+        <v>arrived</v>
+      </c>
+      <c r="L4" t="str">
+        <v>frøen er ankommet</v>
+      </c>
+      <c r="M4" t="str">
+        <v>(6) Facebook</v>
+      </c>
+      <c r="N4" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O4" t="str">
+        <v>https://www.facebook.com/#:~:text=ankommet</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "samtykke" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -88,106 +88,46 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -195,66 +135,27 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -263,143 +164,36 @@
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -760,9 +554,95 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ea9acb4c-4872-4f3e-9fe2-a75c7b9da9a1</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="C5" t="str">
+        <v>samtykke</v>
+      </c>
+      <c r="D5" t="str">
+        <v>samtykke</v>
+      </c>
+      <c r="E5" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F5" t="str">
+        <v>et</v>
+      </c>
+      <c r="G5" t="str">
+        <v>-t</v>
+      </c>
+      <c r="H5" t="str">
+        <v>[ˈsɑmˌtygə]</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://static.ordnet.dk/mp3/11044/11044819_1.mp3</v>
+      </c>
+      <c r="J5" t="str">
+        <v>det at give sin tilladelse til et forslag, en anmodning, en ordning el.lign. især i juridiske sammenhænge</v>
+      </c>
+      <c r="K5" t="str">
+        <v>consent</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Du skal give samtykke til, at sundhed.dk må hente og vise dig persondata på Journaler.</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Journaler - sundhed.dk</v>
+      </c>
+      <c r="N5" t="str">
+        <v>https://www.sundhed.dk/borger/min-side/min-sundhedsjournal/journal-fra-sygehus/</v>
+      </c>
+      <c r="O5" t="str">
+        <v>https://www.sundhed.dk/borger/min-side/min-sundhedsjournal/journal-fra-sygehus/#:~:text=samtykke</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+      <c r="Z5" t="str">
+        <v/>
+      </c>
+      <c r="AA5" t="str">
+        <v/>
+      </c>
+      <c r="AB5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "tilladt" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AB6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -640,9 +640,95 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>e395ff76-4a0f-4c96-8c08-f2eded01bd0f</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C6" t="str">
+        <v>tilladt</v>
+      </c>
+      <c r="D6" t="str">
+        <v>tillade</v>
+      </c>
+      <c r="E6" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>-r, tillod, tilladt</v>
+      </c>
+      <c r="H6" t="str">
+        <v>[ˈteˌlæˀðə]</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://static.ordnet.dk/mp3/12001/12001181_1.mp3</v>
+      </c>
+      <c r="J6" t="str">
+        <v>give lov til; acceptere ofte med henvisning til bestemte love, regler, rettigheder osv.</v>
+      </c>
+      <c r="K6" t="str">
+        <v>allowed</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Må man "drafte" til ALSSUNDMAN? - ALSSUNDMAN er et non-draft race. Det er ikke tilladt at ligge på hjul på cykeldelen. 12-meter-reglen skal overholdes.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N6" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O6" t="str">
+        <v>https://alssundman.dk/faq#:~:text=tilladt</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
+      </c>
+      <c r="Y6" t="str">
+        <v/>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
+      </c>
+      <c r="AA6" t="str">
+        <v/>
+      </c>
+      <c r="AB6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "præmier" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB6"/>
+  <dimension ref="A1:AB7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -726,9 +726,95 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>133bddac-5ab1-4874-b15d-43e0888a8dc8</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C7" t="str">
+        <v>præmier</v>
+      </c>
+      <c r="D7" t="str">
+        <v>præmie</v>
+      </c>
+      <c r="E7" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F7" t="str">
+        <v>en</v>
+      </c>
+      <c r="G7" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H7" t="str">
+        <v>[ˈpʁεːmjə]</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://static.ordnet.dk/mp3/11041/11041293_1.mp3</v>
+      </c>
+      <c r="J7" t="str">
+        <v>belønning (fx penge, et trofæ eller en medalje) som gives til den eller de deltagere der klarer sig bedst i en konkurrence, eller til en person der har ydet en særlig præstation</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Prizes</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Er der præmier til nr. 1,2 og 3? - Der er præmier til hhv. 1.,2., og 3. pladsen i herre- og damerækken på duatlon, AM kort og AM lang.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N7" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O7" t="str">
+        <v>https://alssundman.dk/faq#:~:text=pr%C3%A6mier</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+      <c r="X7" t="str">
+        <v/>
+      </c>
+      <c r="Y7" t="str">
+        <v/>
+      </c>
+      <c r="Z7" t="str">
+        <v/>
+      </c>
+      <c r="AA7" t="str">
+        <v/>
+      </c>
+      <c r="AB7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "øverst" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB7"/>
+  <dimension ref="A1:AB8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -812,9 +812,95 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>78dd3609-e754-4059-a33c-27fd45628daa</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C8" t="str">
+        <v>øverst</v>
+      </c>
+      <c r="D8" t="str">
+        <v>øverst</v>
+      </c>
+      <c r="E8" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>-, -e, som prædikativ: -</v>
+      </c>
+      <c r="H8" t="str">
+        <v>[ˈøwˀʌsd]</v>
+      </c>
+      <c r="I8" t="str">
+        <v>https://static.ordnet.dk/mp3/12008/12008435_1.mp3</v>
+      </c>
+      <c r="J8" t="str">
+        <v>beliggende højest eller meget højt oppe</v>
+      </c>
+      <c r="K8" t="str">
+        <v>upper</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Må jeg deltage på en gammel havelåge, MTB eller gravel cykel? - Det er ikke et krav at man skal cykle på en racer- eller triatloncykel. Cyklen skal overholde kravene fra Triatlon Danmarks konkurrenceregler. (se øverst på siden)</v>
+      </c>
+      <c r="M8" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N8" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O8" t="str">
+        <v>https://alssundman.dk/faq#:~:text=%C3%B8verst</v>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+      <c r="Z8" t="str">
+        <v/>
+      </c>
+      <c r="AA8" t="str">
+        <v/>
+      </c>
+      <c r="AB8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "bevare roen" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB8"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -907,30 +907,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:V2"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1001,9 +1001,77 @@
         <v>Lapses_EN</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>a4be3f33-c5e0-4a35-a584-a0c3420c1f2d</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C2" t="str">
+        <v>bevare roen</v>
+      </c>
+      <c r="D2" t="str">
+        <v>bevare=preserve · roen=the calm</v>
+      </c>
+      <c r="E2" t="str">
+        <v>stay calm</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Hvad skal jeg gøre hvis jeg ser en ulykke? - Hvis der sker en ulykke, er det vigtigt at bevare roen. Du skal selv vurdere hvor alvorligt situationen er. Hvis det er alvorligt og du er den der er tættest på ulykken, skal du stoppe og hjælpe personen indtil der er anden hjælp til stede. Hvis du fortsætter, skal du informere om ulykken ved næste depot eller flagpost.</v>
+      </c>
+      <c r="G2" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://alssundman.dk/faq#:~:text=bevare%20roen</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "vurdere" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB8"/>
+  <dimension ref="A1:AB9"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -898,9 +898,95 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>bd825186-b992-4ff8-b3c1-7457203b82df</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C9" t="str">
+        <v>vurdere</v>
+      </c>
+      <c r="D9" t="str">
+        <v>vurdere</v>
+      </c>
+      <c r="E9" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H9" t="str">
+        <v>[vuɐ̯ˈdeˀʌ]</v>
+      </c>
+      <c r="I9" t="str">
+        <v>https://static.ordnet.dk/mp3/12007/12007388_1.mp3</v>
+      </c>
+      <c r="J9" t="str">
+        <v>anslå eller fastsætte en bestemt pengemæssig værdi af noget, fx et maleri eller en bolig</v>
+      </c>
+      <c r="K9" t="str">
+        <v>assess</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Hvad skal jeg gøre hvis jeg ser en ulykke? - Hvis der sker en ulykke, er det vigtigt at bevare roen. Du skal selv vurdere hvor alvorligt situationen er. Hvis det er alvorligt og du er den der er tættest på ulykken, skal du stoppe og hjælpe personen indtil der er anden hjælp til stede. Hvis du fortsætter, skal du informere om ulykken ved næste depot eller flagpost.</v>
+      </c>
+      <c r="M9" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N9" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O9" t="str">
+        <v>https://alssundman.dk/faq#:~:text=vurdere</v>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+      <c r="X9" t="str">
+        <v/>
+      </c>
+      <c r="Y9" t="str">
+        <v/>
+      </c>
+      <c r="Z9" t="str">
+        <v/>
+      </c>
+      <c r="AA9" t="str">
+        <v/>
+      </c>
+      <c r="AB9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -909,28 +995,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add phrase "går i stykker" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB9"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -993,30 +993,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1155,9 +1155,77 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>4f907ed4-5118-44f0-9aa9-5c66b39fa055</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C3" t="str">
+        <v>går i stykker</v>
+      </c>
+      <c r="D3" t="str">
+        <v>går=going · i=in · stykker=Pieces</v>
+      </c>
+      <c r="E3" t="str">
+        <v>break</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Hvis min cykel går i stykker imens jeg cykler, kan jeg så blive hentet? - Hvis din cykel går i stykker ude på cykelruten og du ikke kan reparere din cykel på stedet, skal du gå hen til de næste flagpost eller til næste depot og informere dem om situationen. De frivillige hjælpere, dommere eller vores Technical Officials ude på ruten kan så kontakte en stævneansvarlig som kan arrangere transport tilbage til stævnepladsen.</v>
+      </c>
+      <c r="G3" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="H3" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://alssundman.dk/faq#:~:text=g%C3%A5r%20i%20stykker</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "imens" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB9"/>
+  <dimension ref="A1:AB10"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -984,9 +984,95 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>6e8b22f4-ec94-4c64-885b-8da51cd5813c</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C10" t="str">
+        <v>imens</v>
+      </c>
+      <c r="D10" t="str">
+        <v>imens</v>
+      </c>
+      <c r="E10" t="str">
+        <v>adverbium</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>[iˈmεnˀs]</v>
+      </c>
+      <c r="I10" t="str">
+        <v>https://static.ordnet.dk/mp3/11023/11023005_1.mp3</v>
+      </c>
+      <c r="J10" t="str">
+        <v>på samme tid som noget andet foregår; samtidig</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Meanwhile</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Hvis min cykel går i stykker imens jeg cykler, kan jeg så blive hentet? - Hvis din cykel går i stykker ude på cykelruten og du ikke kan reparere din cykel på stedet, skal du gå hen til de næste flagpost eller til næste depot og informere dem om situationen. De frivillige hjælpere, dommere eller vores Technical Officials ude på ruten kan så kontakte en stævneansvarlig som kan arrangere transport tilbage til stævnepladsen.</v>
+      </c>
+      <c r="M10" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N10" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O10" t="str">
+        <v>https://alssundman.dk/faq#:~:text=imens</v>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v/>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
+      </c>
+      <c r="AA10" t="str">
+        <v/>
+      </c>
+      <c r="AB10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -995,28 +1081,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V3"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "hentet" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB10"/>
+  <dimension ref="A1:AB11"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1070,9 +1070,95 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>94825bca-7a9f-49f6-880b-2160d8249556</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C11" t="str">
+        <v>hentet</v>
+      </c>
+      <c r="D11" t="str">
+        <v>hente</v>
+      </c>
+      <c r="E11" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H11" t="str">
+        <v>[ˈhεndə]</v>
+      </c>
+      <c r="I11" t="str">
+        <v>https://static.ordnet.dk/mp3/11020/11020472_1.mp3</v>
+      </c>
+      <c r="J11" t="str">
+        <v>tage et bestemt sted hen for at bringe nogen eller noget med sig tilbage</v>
+      </c>
+      <c r="K11" t="str">
+        <v>retrieved</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Hvis min cykel går i stykker imens jeg cykler, kan jeg så blive hentet? - Hvis din cykel går i stykker ude på cykelruten og du ikke kan reparere din cykel på stedet, skal du gå hen til de næste flagpost eller til næste depot og informere dem om situationen. De frivillige hjælpere, dommere eller vores Technical Officials ude på ruten kan så kontakte en stævneansvarlig som kan arrangere transport tilbage til stævnepladsen.</v>
+      </c>
+      <c r="M11" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N11" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O11" t="str">
+        <v>https://alssundman.dk/faq#:~:text=hentet</v>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
+      <c r="Y11" t="str">
+        <v/>
+      </c>
+      <c r="Z11" t="str">
+        <v/>
+      </c>
+      <c r="AA11" t="str">
+        <v/>
+      </c>
+      <c r="AB11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "ansvarlig" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB11"/>
+  <dimension ref="A1:AB12"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1156,9 +1156,95 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>b770b220-0647-4499-afec-09297bc87034</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C12" t="str">
+        <v>ansvarlig</v>
+      </c>
+      <c r="D12" t="str">
+        <v>ansvarlig</v>
+      </c>
+      <c r="E12" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H12" t="str">
+        <v>[anˈsvɑˀli]</v>
+      </c>
+      <c r="I12" t="str">
+        <v>https://static.ordnet.dk/mp3/11001/11001994_1.mp3</v>
+      </c>
+      <c r="J12" t="str">
+        <v>som har ansvar for en bestemt aktivitet (eller person), og som kan drages til ansvar hvis noget går galt</v>
+      </c>
+      <c r="K12" t="str">
+        <v>responsible</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Hvis min cykel går i stykker imens jeg cykler, kan jeg så blive hentet? - Hvis din cykel går i stykker ude på cykelruten og du ikke kan reparere din cykel på stedet, skal du gå hen til de næste flagpost eller til næste depot og informere dem om situationen. De frivillige hjælpere, dommere eller vores Technical Officials ude på ruten kan så kontakte en stævneansvarlig som kan arrangere transport tilbage til stævnepladsen.</v>
+      </c>
+      <c r="M12" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N12" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O12" t="str">
+        <v>https://alssundman.dk/faq#:~:text=ansvarlig</v>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
+      </c>
+      <c r="X12" t="str">
+        <v/>
+      </c>
+      <c r="Y12" t="str">
+        <v/>
+      </c>
+      <c r="Z12" t="str">
+        <v/>
+      </c>
+      <c r="AA12" t="str">
+        <v/>
+      </c>
+      <c r="AB12" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "stævne" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AB13"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1242,9 +1242,95 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>c919541e-3aff-48e4-b834-9017654058b6</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C13" t="str">
+        <v>stævne</v>
+      </c>
+      <c r="D13" t="str">
+        <v>stævne</v>
+      </c>
+      <c r="E13" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F13" t="str">
+        <v>et</v>
+      </c>
+      <c r="G13" t="str">
+        <v>-t, -r, -rne</v>
+      </c>
+      <c r="H13" t="str">
+        <v>[ˈsdεwnə]</v>
+      </c>
+      <c r="I13" t="str">
+        <v>https://static.ordnet.dk/mp3/11051/11051121_1.mp3</v>
+      </c>
+      <c r="J13" t="str">
+        <v>arrangement hvor mange mennesker, ofte fra forskellige egne, mødes for at overvære eller deltage i fx sportskonkurrencer, øvelser eller opvisninger</v>
+      </c>
+      <c r="K13" t="str">
+        <v>convention</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Hvis min cykel går i stykker imens jeg cykler, kan jeg så blive hentet? - Hvis din cykel går i stykker ude på cykelruten og du ikke kan reparere din cykel på stedet, skal du gå hen til de næste flagpost eller til næste depot og informere dem om situationen. De frivillige hjælpere, dommere eller vores Technical Officials ude på ruten kan så kontakte en stævneansvarlig som kan arrangere transport tilbage til stævnepladsen.</v>
+      </c>
+      <c r="M13" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N13" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O13" t="str">
+        <v>https://alssundman.dk/faq#:~:text=st%C3%A6vne</v>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v/>
+      </c>
+      <c r="X13" t="str">
+        <v/>
+      </c>
+      <c r="Y13" t="str">
+        <v/>
+      </c>
+      <c r="Z13" t="str">
+        <v/>
+      </c>
+      <c r="AA13" t="str">
+        <v/>
+      </c>
+      <c r="AB13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "afvikle" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB13"/>
+  <dimension ref="A1:AB14"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1328,9 +1328,95 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>4d9405f3-0704-4a3a-9382-9524ea247725</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C14" t="str">
+        <v>afvikle</v>
+      </c>
+      <c r="D14" t="str">
+        <v>afvikle</v>
+      </c>
+      <c r="E14" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H14" t="str">
+        <v>[-ˌveglə]</v>
+      </c>
+      <c r="I14" t="str">
+        <v>https://static.ordnet.dk/mp3/11000/11000890_1.mp3</v>
+      </c>
+      <c r="J14" t="str">
+        <v>organisere og gennemføre et arrangement</v>
+      </c>
+      <c r="K14" t="str">
+        <v>settle</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Hvornår åbner tilmeldingen til ALSSUNDMAN? - Efter stævnet går der et par uger indtil vi er færdige med at afvikle det hele. Derefter holder vi et evalueringsmøde i arbejdsgruppen hvor vi også beslutter om vi vil afholde ALSSUNDMAN igen året efter. Som regel åbner vi så tilmeldingen i december.</v>
+      </c>
+      <c r="M14" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N14" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O14" t="str">
+        <v>https://alssundman.dk/faq#:~:text=afvikle</v>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
+      <c r="U14" t="str">
+        <v/>
+      </c>
+      <c r="V14" t="str">
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
+        <v/>
+      </c>
+      <c r="Y14" t="str">
+        <v/>
+      </c>
+      <c r="Z14" t="str">
+        <v/>
+      </c>
+      <c r="AA14" t="str">
+        <v/>
+      </c>
+      <c r="AB14" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "regel" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB14"/>
+  <dimension ref="A1:AB15"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1414,9 +1414,95 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>293991e0-0fdf-453a-94a9-0922cc2271eb</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C15" t="str">
+        <v>regel</v>
+      </c>
+      <c r="D15" t="str">
+        <v>regel</v>
+      </c>
+      <c r="E15" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F15" t="str">
+        <v>en</v>
+      </c>
+      <c r="G15" t="str">
+        <v>reglen (eller uofficiel form: -en), regler, reglerne Se bøjning i skema</v>
+      </c>
+      <c r="H15" t="str">
+        <v>[ˈʁεjˀəl]</v>
+      </c>
+      <c r="I15" t="str">
+        <v>https://static.ordnet.dk/mp3/11042/11042476_1.mp3</v>
+      </c>
+      <c r="J15" t="str">
+        <v>bestemmelse om hvordan noget skal foregå, eller hvordan man skal forholde sig i en bestemt situation</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Rule</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Hvornår åbner tilmeldingen til ALSSUNDMAN? - Efter stævnet går der et par uger indtil vi er færdige med at afvikle det hele. Derefter holder vi et evalueringsmøde i arbejdsgruppen hvor vi også beslutter om vi vil afholde ALSSUNDMAN igen året efter. Som regel åbner vi så tilmeldingen i december.</v>
+      </c>
+      <c r="M15" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N15" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O15" t="str">
+        <v>https://alssundman.dk/faq#:~:text=regel</v>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
+        <v/>
+      </c>
+      <c r="X15" t="str">
+        <v/>
+      </c>
+      <c r="Y15" t="str">
+        <v/>
+      </c>
+      <c r="Z15" t="str">
+        <v/>
+      </c>
+      <c r="AA15" t="str">
+        <v/>
+      </c>
+      <c r="AB15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "beslutter" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB15"/>
+  <dimension ref="A1:AB16"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1500,9 +1500,95 @@
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>e7faf51e-441a-45b8-8da4-8afdb60eab47</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C16" t="str">
+        <v>beslutter</v>
+      </c>
+      <c r="D16" t="str">
+        <v>beslutter</v>
+      </c>
+      <c r="E16" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F16" t="str">
+        <v>en</v>
+      </c>
+      <c r="G16" t="str">
+        <v>-en, -e, -ne</v>
+      </c>
+      <c r="H16" t="str">
+        <v>[beˈsludʌ]</v>
+      </c>
+      <c r="I16" t="str">
+        <v>https://static.ordnet.dk/mp3/40000/40000324_1.mp3</v>
+      </c>
+      <c r="J16" t="str">
+        <v>person der træffer beslutninger</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Deciding</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Hvornår åbner tilmeldingen til ALSSUNDMAN? - Efter stævnet går der et par uger indtil vi er færdige med at afvikle det hele. Derefter holder vi et evalueringsmøde i arbejdsgruppen hvor vi også beslutter om vi vil afholde ALSSUNDMAN igen året efter. Som regel åbner vi så tilmeldingen i december.</v>
+      </c>
+      <c r="M16" t="str">
+        <v>FAQ</v>
+      </c>
+      <c r="N16" t="str">
+        <v>https://alssundman.dk/faq</v>
+      </c>
+      <c r="O16" t="str">
+        <v>https://alssundman.dk/faq#:~:text=beslutter</v>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str">
+        <v/>
+      </c>
+      <c r="V16" t="str">
+        <v/>
+      </c>
+      <c r="W16" t="str">
+        <v/>
+      </c>
+      <c r="X16" t="str">
+        <v/>
+      </c>
+      <c r="Y16" t="str">
+        <v/>
+      </c>
+      <c r="Z16" t="str">
+        <v/>
+      </c>
+      <c r="AA16" t="str">
+        <v/>
+      </c>
+      <c r="AB16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "øget" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AB17"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1586,9 +1586,95 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>1d146782-f430-4a3b-8bee-73dcf985f1b2</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C17" t="str">
+        <v>øget</v>
+      </c>
+      <c r="D17" t="str">
+        <v>øg</v>
+      </c>
+      <c r="E17" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F17" t="str">
+        <v>et</v>
+      </c>
+      <c r="G17" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H17" t="str">
+        <v>[ˈøˀj]</v>
+      </c>
+      <c r="I17" t="str">
+        <v>https://static.ordnet.dk/mp3/12008/12008194_1.mp3</v>
+      </c>
+      <c r="J17" t="str">
+        <v>gammel, udslidt hest</v>
+      </c>
+      <c r="K17" t="str">
+        <v>increased</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Ifølge beretningen anerkender Forsvarsministeriet, at der ikke var dokumentation for behovet for de tusindvis af ekstra schweizerknive. Ministeriet oplyser dog, »at købet skyldes et øget behov for udrustning til personalet«.</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="N17" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="O17" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=%C3%B8get</v>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17" t="str">
+        <v/>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str">
+        <v/>
+      </c>
+      <c r="V17" t="str">
+        <v/>
+      </c>
+      <c r="W17" t="str">
+        <v/>
+      </c>
+      <c r="X17" t="str">
+        <v/>
+      </c>
+      <c r="Y17" t="str">
+        <v/>
+      </c>
+      <c r="Z17" t="str">
+        <v/>
+      </c>
+      <c r="AA17" t="str">
+        <v/>
+      </c>
+      <c r="AB17" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "udrustning" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB17"/>
+  <dimension ref="A1:AB18"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1672,9 +1672,95 @@
         <v/>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>9c247006-2823-470e-9723-43c9ee4d023f</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C18" t="str">
+        <v>udrustning</v>
+      </c>
+      <c r="D18" t="str">
+        <v>udrustning</v>
+      </c>
+      <c r="E18" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F18" t="str">
+        <v>en</v>
+      </c>
+      <c r="G18" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H18" t="str">
+        <v>[-ˌʁɔsdneŋ]</v>
+      </c>
+      <c r="I18" t="str">
+        <v>https://static.ordnet.dk/mp3/12004/12004058_1.mp3</v>
+      </c>
+      <c r="J18" t="str">
+        <v>udstyr, våben el.lign. som nogen er forsynet med til et bestemt formål</v>
+      </c>
+      <c r="K18" t="str">
+        <v>fitting</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Ifølge beretningen anerkender Forsvarsministeriet, at der ikke var dokumentation for behovet for de tusindvis af ekstra schweizerknive. Ministeriet oplyser dog, »at købet skyldes et øget behov for udrustning til personalet«.</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="N18" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="O18" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=udrustning</v>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str">
+        <v/>
+      </c>
+      <c r="V18" t="str">
+        <v/>
+      </c>
+      <c r="W18" t="str">
+        <v/>
+      </c>
+      <c r="X18" t="str">
+        <v/>
+      </c>
+      <c r="Y18" t="str">
+        <v/>
+      </c>
+      <c r="Z18" t="str">
+        <v/>
+      </c>
+      <c r="AA18" t="str">
+        <v/>
+      </c>
+      <c r="AB18" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB18"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update translation of "udrustning" in Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB18"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1704,7 +1704,7 @@
         <v>udstyr, våben el.lign. som nogen er forsynet med til et bestemt formål</v>
       </c>
       <c r="K18" t="str">
-        <v>fitting</v>
+        <v>fitting/outfitting</v>
       </c>
       <c r="L18" t="str">
         <v>Ifølge beretningen anerkender Forsvarsministeriet, at der ikke var dokumentation for behovet for de tusindvis af ekstra schweizerknive. Ministeriet oplyser dog, »at købet skyldes et øget behov for udrustning til personalet«.</v>

</xml_diff>

<commit_message>
Add word "lås" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB18"/>
+  <dimension ref="A1:AB19"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1758,9 +1758,95 @@
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>d40508d7-f2ce-42e8-99b7-17ad25fb58cd</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-08-23</v>
+      </c>
+      <c r="C19" t="str">
+        <v>lås</v>
+      </c>
+      <c r="D19" t="str">
+        <v>lås</v>
+      </c>
+      <c r="E19" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F19" t="str">
+        <v>en</v>
+      </c>
+      <c r="G19" t="str">
+        <v>-en, -e, -ene</v>
+      </c>
+      <c r="H19" t="str">
+        <v>[ˈlɔˀs]</v>
+      </c>
+      <c r="I19" t="str">
+        <v>https://static.ordnet.dk/mp3/11031/11031954_1.mp3</v>
+      </c>
+      <c r="J19" t="str">
+        <v>mekanisme der skal sikre at adgangen til noget holdes afspærret for uvedkommende; kan fx bestå af en bevægelig metalstang (rigel) der skydes ind i et hul ved hjælp af en tilhørende nøgle, hvorefter låsen kun kan åbnes med nøglen</v>
+      </c>
+      <c r="K19" t="str">
+        <v>lock</v>
+      </c>
+      <c r="L19" t="str">
+        <v>COMPANION M2.0 Størrelse XL (Hjulstr: 29″) - Farve Petroleumsblå Gear: Type &amp; Antal Shimano Tourney - 21 gear Købt 2. marts 2024 Med kvittering og lås. See less</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Marketplace - Cykel Companion M2.0 | Facebook</v>
+      </c>
+      <c r="N19" t="str">
+        <v>https://www.facebook.com/marketplace/item/2264869994334498?ref=search&amp;referral_code=null&amp;referral_story_type=post&amp;tracking=browse_serp%3A65c4d7f8-925b-432a-9f5b-2a17767b70a9</v>
+      </c>
+      <c r="O19" t="str">
+        <v>https://www.facebook.com/marketplace/item/2264869994334498?ref=search&amp;referral_code=null&amp;referral_story_type=post&amp;tracking=browse_serp%3A65c4d7f8-925b-432a-9f5b-2a17767b70a9#:~:text=l%C3%A5s</v>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str">
+        <v/>
+      </c>
+      <c r="V19" t="str">
+        <v/>
+      </c>
+      <c r="W19" t="str">
+        <v/>
+      </c>
+      <c r="X19" t="str">
+        <v/>
+      </c>
+      <c r="Y19" t="str">
+        <v/>
+      </c>
+      <c r="Z19" t="str">
+        <v/>
+      </c>
+      <c r="AA19" t="str">
+        <v/>
+      </c>
+      <c r="AB19" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "beskyttelse" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB19"/>
+  <dimension ref="A1:AB20"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1844,9 +1844,95 @@
         <v/>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>87467a7f-ff4c-429d-a450-c067e9959997</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C20" t="str">
+        <v>beskyttelse</v>
+      </c>
+      <c r="D20" t="str">
+        <v>beskyttelse</v>
+      </c>
+      <c r="E20" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F20" t="str">
+        <v>en</v>
+      </c>
+      <c r="G20" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H20" t="str">
+        <v>[beˈsgødəlsə]</v>
+      </c>
+      <c r="I20" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004240_1.mp3</v>
+      </c>
+      <c r="J20" t="str">
+        <v>det at beskytte eller blive beskyttet</v>
+      </c>
+      <c r="K20" t="str">
+        <v>protection</v>
+      </c>
+      <c r="L20" t="str">
+        <v>dyrenesbeskyttelse</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Instagram</v>
+      </c>
+      <c r="N20" t="str">
+        <v>https://www.instagram.com/</v>
+      </c>
+      <c r="O20" t="str">
+        <v>https://www.instagram.com/#:~:text=beskyttelse</v>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str">
+        <v/>
+      </c>
+      <c r="V20" t="str">
+        <v/>
+      </c>
+      <c r="W20" t="str">
+        <v/>
+      </c>
+      <c r="X20" t="str">
+        <v/>
+      </c>
+      <c r="Y20" t="str">
+        <v/>
+      </c>
+      <c r="Z20" t="str">
+        <v/>
+      </c>
+      <c r="AA20" t="str">
+        <v/>
+      </c>
+      <c r="AB20" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "førte" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB20"/>
+  <dimension ref="A1:AB21"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1930,9 +1930,95 @@
         <v/>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>877f54ca-3aca-4523-91fe-5a16b8c97b6b</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C21" t="str">
+        <v>førte</v>
+      </c>
+      <c r="D21" t="str">
+        <v>føre</v>
+      </c>
+      <c r="E21" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v>-r, førte, ført</v>
+      </c>
+      <c r="H21" t="str">
+        <v>[ˈføːʌ]</v>
+      </c>
+      <c r="I21" t="str">
+        <v>https://static.ordnet.dk/mp3/11016/11016882_1.mp3</v>
+      </c>
+      <c r="J21" t="str">
+        <v>transportere eller flytte i en bestemt retning eller et bestemt sted hen</v>
+      </c>
+      <c r="K21" t="str">
+        <v>led</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Præcis hvem knivene skulle tildeles, hvad der førte til fejlkøbet, og hvor meget det har kostet, fremgår ikke.</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="N21" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="O21" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=f%C3%B8rte</v>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
+      <c r="S21" t="str">
+        <v/>
+      </c>
+      <c r="T21" t="str">
+        <v/>
+      </c>
+      <c r="U21" t="str">
+        <v/>
+      </c>
+      <c r="V21" t="str">
+        <v/>
+      </c>
+      <c r="W21" t="str">
+        <v/>
+      </c>
+      <c r="X21" t="str">
+        <v/>
+      </c>
+      <c r="Y21" t="str">
+        <v/>
+      </c>
+      <c r="Z21" t="str">
+        <v/>
+      </c>
+      <c r="AA21" t="str">
+        <v/>
+      </c>
+      <c r="AB21" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "mangelfuld" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB21"/>
+  <dimension ref="A1:AB22"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2016,9 +2016,95 @@
         <v/>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>3741082b-bf56-4c1e-bc3c-18c84b8666a5</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C22" t="str">
+        <v>mangelfuld</v>
+      </c>
+      <c r="D22" t="str">
+        <v>mangelfuld</v>
+      </c>
+      <c r="E22" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v>https://static.ordnet.dk/mp3/11032/11032347_1.mp3</v>
+      </c>
+      <c r="J22" t="str">
+        <v>som har mangler; som ikke er fuldkommen</v>
+      </c>
+      <c r="K22" t="str">
+        <v>defective</v>
+      </c>
+      <c r="L22" t="str">
+        <v>I beretningen får Forsvarsministeriet også kritik for sit indkøb generelt. En gennemgang af indkøb fra 2023 til 2025 viser, at 27 procent af Forsvarets indkøb enten helt mangler eller har en mangelfuld afdækning af behovet.</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="N22" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="O22" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=mangelfuld</v>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
+      <c r="T22" t="str">
+        <v/>
+      </c>
+      <c r="U22" t="str">
+        <v/>
+      </c>
+      <c r="V22" t="str">
+        <v/>
+      </c>
+      <c r="W22" t="str">
+        <v/>
+      </c>
+      <c r="X22" t="str">
+        <v/>
+      </c>
+      <c r="Y22" t="str">
+        <v/>
+      </c>
+      <c r="Z22" t="str">
+        <v/>
+      </c>
+      <c r="AA22" t="str">
+        <v/>
+      </c>
+      <c r="AB22" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "afdækning" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB22"/>
+  <dimension ref="A1:AB23"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2102,9 +2102,95 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>44e9f1a8-d361-4346-8362-4e8456d334b6</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C23" t="str">
+        <v>afdækning</v>
+      </c>
+      <c r="D23" t="str">
+        <v>afdækning</v>
+      </c>
+      <c r="E23" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F23" t="str">
+        <v>en</v>
+      </c>
+      <c r="G23" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v>https://static.ordnet.dk/mp3/11000/11000339_1.mp3</v>
+      </c>
+      <c r="J23" t="str">
+        <v>det at dække noget til for at beskytte det mod vand, snavs el.lign.</v>
+      </c>
+      <c r="K23" t="str">
+        <v>cover</v>
+      </c>
+      <c r="L23" t="str">
+        <v>I beretningen får Forsvarsministeriet også kritik for sit indkøb generelt. En gennemgang af indkøb fra 2023 til 2025 viser, at 27 procent af Forsvarets indkøb enten helt mangler eller har en mangelfuld afdækning af behovet.</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="N23" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="O23" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=afd%C3%A6kning</v>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v/>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <v/>
+      </c>
+      <c r="Y23" t="str">
+        <v/>
+      </c>
+      <c r="Z23" t="str">
+        <v/>
+      </c>
+      <c r="AA23" t="str">
+        <v/>
+      </c>
+      <c r="AB23" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Samtidig" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB23"/>
+  <dimension ref="A1:AB24"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2188,9 +2188,95 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>7334c944-f28b-48e7-80ed-49259f26e2e1</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Samtidig</v>
+      </c>
+      <c r="D24" t="str">
+        <v>samtidig</v>
+      </c>
+      <c r="E24" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v>-t, -e som adverbium: -t eller -, for eksempel “de ankom samtidig(t)”</v>
+      </c>
+      <c r="H24" t="str">
+        <v>[ˈsɑmˌtiðˀi]</v>
+      </c>
+      <c r="I24" t="str">
+        <v>https://static.ordnet.dk/mp3/11044/11044814_1.mp3</v>
+      </c>
+      <c r="J24" t="str">
+        <v>som foregår eller findes på (omtrent) samme tid som noget andet</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Simultaneous</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Samtidig mangler der også dokumentation for, at ministeriet har undersøgt prisniveau, leveringsvilkår eller alternative leverandører i 73 procent af købene.</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="N24" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="O24" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=Samtidig</v>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v/>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
+      <c r="W24" t="str">
+        <v/>
+      </c>
+      <c r="X24" t="str">
+        <v/>
+      </c>
+      <c r="Y24" t="str">
+        <v/>
+      </c>
+      <c r="Z24" t="str">
+        <v/>
+      </c>
+      <c r="AA24" t="str">
+        <v/>
+      </c>
+      <c r="AB24" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "undersøgt" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB24"/>
+  <dimension ref="A1:AB25"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2274,9 +2274,95 @@
         <v/>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>42a36227-205a-4e67-93ad-0303c33384a4</v>
+      </c>
+      <c r="B25" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C25" t="str">
+        <v>undersøgt</v>
+      </c>
+      <c r="D25" t="str">
+        <v>undersøge</v>
+      </c>
+      <c r="E25" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v>-r, ..søgte, ..søgt</v>
+      </c>
+      <c r="H25" t="str">
+        <v>[ˈɔnʌˌsøˀjə]</v>
+      </c>
+      <c r="I25" t="str">
+        <v>https://static.ordnet.dk/mp3/12004/12004873_1.mp3</v>
+      </c>
+      <c r="J25" t="str">
+        <v>underkaste noget, fx en genstand, et materiale, et område eller en organisme, en nøje og detaljeret gennemgang, med henblik på at finde frem til og opnå sikker viden om dets beskaffenhed, sammensætning, struktur osv. ofte på basis af en bestemt syste</v>
+      </c>
+      <c r="K25" t="str">
+        <v>investigated</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Samtidig mangler der også dokumentation for, at ministeriet har undersøgt prisniveau, leveringsvilkår eller alternative leverandører i 73 procent af købene.</v>
+      </c>
+      <c r="M25" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="N25" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="O25" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=unders%C3%B8gt</v>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
+      <c r="S25" t="str">
+        <v/>
+      </c>
+      <c r="T25" t="str">
+        <v/>
+      </c>
+      <c r="U25" t="str">
+        <v/>
+      </c>
+      <c r="V25" t="str">
+        <v/>
+      </c>
+      <c r="W25" t="str">
+        <v/>
+      </c>
+      <c r="X25" t="str">
+        <v/>
+      </c>
+      <c r="Y25" t="str">
+        <v/>
+      </c>
+      <c r="Z25" t="str">
+        <v/>
+      </c>
+      <c r="AA25" t="str">
+        <v/>
+      </c>
+      <c r="AB25" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "vilkår" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB25"/>
+  <dimension ref="A1:AB26"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2360,9 +2360,95 @@
         <v/>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>7537d9d8-7248-4e49-8694-e39d5318a430</v>
+      </c>
+      <c r="B26" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C26" t="str">
+        <v>vilkår</v>
+      </c>
+      <c r="D26" t="str">
+        <v>vilkår</v>
+      </c>
+      <c r="E26" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F26" t="str">
+        <v>et</v>
+      </c>
+      <c r="G26" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H26" t="str">
+        <v>[ˈvilˌkɒˀ]</v>
+      </c>
+      <c r="I26" t="str">
+        <v>https://static.ordnet.dk/mp3/12006/12006771_1.mp3</v>
+      </c>
+      <c r="J26" t="str">
+        <v>ydre omstændighed som er bestemmende for hvordan noget skal foregå, udvikle sig el.lign. om fx de samfundsmæssige forhold som man lever under</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Terms</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Samtidig mangler der også dokumentation for, at ministeriet har undersøgt prisniveau, leveringsvilkår eller alternative leverandører i 73 procent af købene.</v>
+      </c>
+      <c r="M26" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="N26" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="O26" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=vilk%C3%A5r</v>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26" t="str">
+        <v/>
+      </c>
+      <c r="T26" t="str">
+        <v/>
+      </c>
+      <c r="U26" t="str">
+        <v/>
+      </c>
+      <c r="V26" t="str">
+        <v/>
+      </c>
+      <c r="W26" t="str">
+        <v/>
+      </c>
+      <c r="X26" t="str">
+        <v/>
+      </c>
+      <c r="Y26" t="str">
+        <v/>
+      </c>
+      <c r="Z26" t="str">
+        <v/>
+      </c>
+      <c r="AA26" t="str">
+        <v/>
+      </c>
+      <c r="AB26" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB26"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "leverandører" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB26"/>
+  <dimension ref="A1:AB27"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2446,9 +2446,95 @@
         <v/>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>f34aa9b7-d20c-40b5-a304-1af0aec943e7</v>
+      </c>
+      <c r="B27" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C27" t="str">
+        <v>leverandører</v>
+      </c>
+      <c r="D27" t="str">
+        <v>leverandør</v>
+      </c>
+      <c r="E27" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F27" t="str">
+        <v>en</v>
+      </c>
+      <c r="G27" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H27" t="str">
+        <v>[levəʁɑnˈdøˀɐ̯]</v>
+      </c>
+      <c r="I27" t="str">
+        <v>https://static.ordnet.dk/mp3/11030/11030265_1.mp3</v>
+      </c>
+      <c r="J27" t="str">
+        <v>firma, handelsmand eller land der regelmæssigt sælger eller eksporterer en (bestemt) vare til en (bestemt) køber</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Suppliers</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Samtidig mangler der også dokumentation for, at ministeriet har undersøgt prisniveau, leveringsvilkår eller alternative leverandører i 73 procent af købene.</v>
+      </c>
+      <c r="M27" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="N27" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="O27" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=leverand%C3%B8rer</v>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+      <c r="T27" t="str">
+        <v/>
+      </c>
+      <c r="U27" t="str">
+        <v/>
+      </c>
+      <c r="V27" t="str">
+        <v/>
+      </c>
+      <c r="W27" t="str">
+        <v/>
+      </c>
+      <c r="X27" t="str">
+        <v/>
+      </c>
+      <c r="Y27" t="str">
+        <v/>
+      </c>
+      <c r="Z27" t="str">
+        <v/>
+      </c>
+      <c r="AA27" t="str">
+        <v/>
+      </c>
+      <c r="AB27" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB27"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "rakt" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB27"/>
+  <dimension ref="A1:AB28"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2532,9 +2532,95 @@
         <v/>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>1370e6a4-df3b-49d6-acda-b2cb3e62a2ec</v>
+      </c>
+      <c r="B28" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C28" t="str">
+        <v>rakt</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v>-r, rakte, rakt</v>
+      </c>
+      <c r="H28" t="str">
+        <v>[ˈʁagə]</v>
+      </c>
+      <c r="I28" t="str">
+        <v>https://static.ordnet.dk/mp3/11044/11044068_1.mp3</v>
+      </c>
+      <c r="J28" t="str">
+        <v>gribe fat om noget med hånden eller hænderne og give det til en anden</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Raked</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Ingeniøren har rakt ud til Forsvarets Materiel- og Indkøbsstyrelse, der ikke har vendt tilbage inden deadline.</v>
+      </c>
+      <c r="M28" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="N28" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="O28" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=rakt</v>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
+      <c r="S28" t="str">
+        <v/>
+      </c>
+      <c r="T28" t="str">
+        <v/>
+      </c>
+      <c r="U28" t="str">
+        <v/>
+      </c>
+      <c r="V28" t="str">
+        <v/>
+      </c>
+      <c r="W28" t="str">
+        <v/>
+      </c>
+      <c r="X28" t="str">
+        <v/>
+      </c>
+      <c r="Y28" t="str">
+        <v/>
+      </c>
+      <c r="Z28" t="str">
+        <v/>
+      </c>
+      <c r="AA28" t="str">
+        <v/>
+      </c>
+      <c r="AB28" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB28"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "rakt ud" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB28"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2627,30 +2627,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V4"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2857,9 +2857,77 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>bb4542b5-264a-4c51-a0fa-2dd715192389</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C4" t="str">
+        <v>rakt ud</v>
+      </c>
+      <c r="D4" t="str">
+        <v>rakt=Raked · ud=out</v>
+      </c>
+      <c r="E4" t="str">
+        <v>reached out</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Ingeniøren har rakt ud til Forsvarets Materiel- og Indkøbsstyrelse, der ikke har vendt tilbage inden deadline.</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Kæmpe regnefejl: Forsvaret har købt 27.000 schweizerknive for meget | Ingeniøren</v>
+      </c>
+      <c r="H4" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://ing.dk/artikel/kaempe-regnefejl-forsvaret-har-koebt-27000-schweizerknive-meget#:~:text=rakt%20ud</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Ledige" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB28"/>
+  <dimension ref="A1:AB29"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2618,9 +2618,95 @@
         <v/>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>db1c6d6a-2297-4a5a-bf4f-2b96722a7504</v>
+      </c>
+      <c r="B29" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Ledige</v>
+      </c>
+      <c r="D29" t="str">
+        <v>ledig</v>
+      </c>
+      <c r="E29" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H29" t="str">
+        <v>[ˈleːði]</v>
+      </c>
+      <c r="I29" t="str">
+        <v>https://static.ordnet.dk/mp3/11030/11030028_1.mp3</v>
+      </c>
+      <c r="J29" t="str">
+        <v>ikke optaget; fri; til rådighed</v>
+      </c>
+      <c r="K29" t="str">
+        <v>vacant</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Ledige stillinger</v>
+      </c>
+      <c r="M29" t="str">
+        <v>Maskiningeniør</v>
+      </c>
+      <c r="N29" t="str">
+        <v>https://www.fmi.dk/da/karriere/ingenior/maskiningenior/</v>
+      </c>
+      <c r="O29" t="str">
+        <v>https://www.fmi.dk/da/karriere/ingenior/maskiningenior/#:~:text=Ledige</v>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R29" t="str">
+        <v/>
+      </c>
+      <c r="S29" t="str">
+        <v/>
+      </c>
+      <c r="T29" t="str">
+        <v/>
+      </c>
+      <c r="U29" t="str">
+        <v/>
+      </c>
+      <c r="V29" t="str">
+        <v/>
+      </c>
+      <c r="W29" t="str">
+        <v/>
+      </c>
+      <c r="X29" t="str">
+        <v/>
+      </c>
+      <c r="Y29" t="str">
+        <v/>
+      </c>
+      <c r="Z29" t="str">
+        <v/>
+      </c>
+      <c r="AA29" t="str">
+        <v/>
+      </c>
+      <c r="AB29" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2629,28 +2715,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V4"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "stillinger" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB29"/>
+  <dimension ref="A1:AB30"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2704,9 +2704,95 @@
         <v/>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>82ed41a4-8ced-4691-a11a-2d6db2795869</v>
+      </c>
+      <c r="B30" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C30" t="str">
+        <v>stillinger</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v>Positions</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Ledige stillinger</v>
+      </c>
+      <c r="M30" t="str">
+        <v>Maskiningeniør</v>
+      </c>
+      <c r="N30" t="str">
+        <v>https://www.fmi.dk/da/karriere/ingenior/maskiningenior/</v>
+      </c>
+      <c r="O30" t="str">
+        <v>https://www.fmi.dk/da/karriere/ingenior/maskiningenior/#:~:text=stillinger</v>
+      </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
+        <v>pending</v>
+      </c>
+      <c r="R30" t="str">
+        <v/>
+      </c>
+      <c r="S30" t="str">
+        <v/>
+      </c>
+      <c r="T30" t="str">
+        <v/>
+      </c>
+      <c r="U30" t="str">
+        <v/>
+      </c>
+      <c r="V30" t="str">
+        <v/>
+      </c>
+      <c r="W30" t="str">
+        <v/>
+      </c>
+      <c r="X30" t="str">
+        <v/>
+      </c>
+      <c r="Y30" t="str">
+        <v/>
+      </c>
+      <c r="Z30" t="str">
+        <v/>
+      </c>
+      <c r="AA30" t="str">
+        <v/>
+      </c>
+      <c r="AB30" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "krus" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB30"/>
+  <dimension ref="A1:AB31"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2790,9 +2790,95 @@
         <v/>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>1de60b9a-939a-4116-8c4a-88154d385378</v>
+      </c>
+      <c r="B31" t="str">
+        <v>2026-08-25</v>
+      </c>
+      <c r="C31" t="str">
+        <v>krus</v>
+      </c>
+      <c r="D31" t="str">
+        <v>krus</v>
+      </c>
+      <c r="E31" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F31" t="str">
+        <v>et</v>
+      </c>
+      <c r="G31" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H31" t="str">
+        <v>[ˈkʁuˀs]</v>
+      </c>
+      <c r="I31" t="str">
+        <v>https://static.ordnet.dk/mp3/11028/11028277_1.mp3</v>
+      </c>
+      <c r="J31" t="str">
+        <v>cylinderformet beholder, som regel med hank, fremstillet af keramik, metal el.lign. og beregnet til at drikke af</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Mug</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Et krus til kaffepausen og dit gode humør!</v>
+      </c>
+      <c r="M31" t="str">
+        <v>Fællesklang Odense</v>
+      </c>
+      <c r="N31" t="str">
+        <v>https://kfum-kfuk.dk/odense/aktiviteter/faellesklang-odense/</v>
+      </c>
+      <c r="O31" t="str">
+        <v>https://kfum-kfuk.dk/odense/aktiviteter/faellesklang-odense/#:~:text=krus</v>
+      </c>
+      <c r="P31" t="str">
+        <v/>
+      </c>
+      <c r="Q31" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R31" t="str">
+        <v/>
+      </c>
+      <c r="S31" t="str">
+        <v/>
+      </c>
+      <c r="T31" t="str">
+        <v/>
+      </c>
+      <c r="U31" t="str">
+        <v/>
+      </c>
+      <c r="V31" t="str">
+        <v/>
+      </c>
+      <c r="W31" t="str">
+        <v/>
+      </c>
+      <c r="X31" t="str">
+        <v/>
+      </c>
+      <c r="Y31" t="str">
+        <v/>
+      </c>
+      <c r="Z31" t="str">
+        <v/>
+      </c>
+      <c r="AA31" t="str">
+        <v/>
+      </c>
+      <c r="AB31" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Forventer" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB31"/>
+  <dimension ref="A1:AB32"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2876,9 +2876,95 @@
         <v/>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>99cc5d28-588f-4375-a0b8-d11fe34e236f</v>
+      </c>
+      <c r="B32" t="str">
+        <v>2026-08-25</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Forventer</v>
+      </c>
+      <c r="D32" t="str">
+        <v>forvente</v>
+      </c>
+      <c r="E32" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H32" t="str">
+        <v>[fʌˈvεnˀdə]</v>
+      </c>
+      <c r="I32" t="str">
+        <v>https://static.ordnet.dk/mp3/11015/11015506_1.mp3</v>
+      </c>
+      <c r="J32" t="str">
+        <v>regne med at noget med en vis sandsynlighed vil ske eller forløbe på en bestemt måde i fremtiden</v>
+      </c>
+      <c r="K32" t="str">
+        <v>expecting</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Forventer du at deltage/deltager du allerede i nogle af foreningens andre aktiviteter? *</v>
+      </c>
+      <c r="M32" t="str">
+        <v>Tilmelding til Fællesklang Odenses efterårssæson 2026 | KFUM og KFUK i Danmark</v>
+      </c>
+      <c r="N32" t="str">
+        <v>https://medlem.kfum-kfuk.dk/en_GB/event/id/942/register?fbclid=IwY2xjawT63m5wZG9mAWV4dG4DYWVtAjEwAGJyaWQRMEJYSGxzNUd2aFZBYmIxQWpzcnRjBmFwcF9pZBAyMjIwMzkxNzg4MjAwODkyAAEecMCmXTbNjtw5jXJEIRp5sTtqUqmLjdFtDKrqdJbdfO2w8UzoA2HtIswZ7sg_aem_-mBQj6FhsjNmQ7z5ueiPIg</v>
+      </c>
+      <c r="O32" t="str">
+        <v>https://medlem.kfum-kfuk.dk/en_GB/event/id/942/register?fbclid=IwY2xjawT63m5wZG9mAWV4dG4DYWVtAjEwAGJyaWQRMEJYSGxzNUd2aFZBYmIxQWpzcnRjBmFwcF9pZBAyMjIwMzkxNzg4MjAwODkyAAEecMCmXTbNjtw5jXJEIRp5sTtqUqmLjdFtDKrqdJbdfO2w8UzoA2HtIswZ7sg_aem_-mBQj6FhsjNmQ7z5ueiPIg#:~:text=Forventer</v>
+      </c>
+      <c r="P32" t="str">
+        <v/>
+      </c>
+      <c r="Q32" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R32" t="str">
+        <v/>
+      </c>
+      <c r="S32" t="str">
+        <v/>
+      </c>
+      <c r="T32" t="str">
+        <v/>
+      </c>
+      <c r="U32" t="str">
+        <v/>
+      </c>
+      <c r="V32" t="str">
+        <v/>
+      </c>
+      <c r="W32" t="str">
+        <v/>
+      </c>
+      <c r="X32" t="str">
+        <v/>
+      </c>
+      <c r="Y32" t="str">
+        <v/>
+      </c>
+      <c r="Z32" t="str">
+        <v/>
+      </c>
+      <c r="AA32" t="str">
+        <v/>
+      </c>
+      <c r="AB32" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB32"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Derudover" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB32"/>
+  <dimension ref="A1:AB33"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2962,9 +2962,95 @@
         <v/>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>bea2cf27-ddb9-41a5-9bec-31b12650657f</v>
+      </c>
+      <c r="B33" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Derudover</v>
+      </c>
+      <c r="D33" t="str">
+        <v>derudover</v>
+      </c>
+      <c r="E33" t="str">
+        <v>adverbium</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v>[ˈdεˀɐ̯uðˌɒwˀʌ]</v>
+      </c>
+      <c r="I33" t="str">
+        <v>https://static.ordnet.dk/mp3/11008/11008835_1.mp3</v>
+      </c>
+      <c r="J33" t="str">
+        <v>ud over det netop nævnte</v>
+      </c>
+      <c r="K33" t="str">
+        <v>In addition</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Undersøgelsen handler om, hvad der er vigtigt i dit arbejdsliv og hvilke IT-virksomheder, der er de mest attraktive. Derudover handler den om brugen af AI på arbejdspladsen. Det tager 8-10 minutter at deltage, afhængig af besvarelsen kan tiden variere.</v>
+      </c>
+      <c r="M33" t="str">
+        <v>Hvad er vigtigtst i dit arbejdsliv? - yihengldavid@gmail.com - Gmail</v>
+      </c>
+      <c r="N33" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
+      </c>
+      <c r="O33" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=Derudover</v>
+      </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R33" t="str">
+        <v/>
+      </c>
+      <c r="S33" t="str">
+        <v/>
+      </c>
+      <c r="T33" t="str">
+        <v/>
+      </c>
+      <c r="U33" t="str">
+        <v/>
+      </c>
+      <c r="V33" t="str">
+        <v/>
+      </c>
+      <c r="W33" t="str">
+        <v/>
+      </c>
+      <c r="X33" t="str">
+        <v/>
+      </c>
+      <c r="Y33" t="str">
+        <v/>
+      </c>
+      <c r="Z33" t="str">
+        <v/>
+      </c>
+      <c r="AA33" t="str">
+        <v/>
+      </c>
+      <c r="AB33" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB33"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "deltage" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB33"/>
+  <dimension ref="A1:AB34"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3048,9 +3048,95 @@
         <v/>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>d6129f35-7b91-493d-b96b-f52edd1f1480</v>
+      </c>
+      <c r="B34" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C34" t="str">
+        <v>deltage</v>
+      </c>
+      <c r="D34" t="str">
+        <v>deltage</v>
+      </c>
+      <c r="E34" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v>-r, deltog, -t</v>
+      </c>
+      <c r="H34" t="str">
+        <v>[ˈdelˌtæˀ]</v>
+      </c>
+      <c r="I34" t="str">
+        <v>https://static.ordnet.dk/mp3/11008/11008669_1.mp3</v>
+      </c>
+      <c r="J34" t="str">
+        <v>være med i en aktivitet</v>
+      </c>
+      <c r="K34" t="str">
+        <v>participate</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Undersøgelsen handler om, hvad der er vigtigt i dit arbejdsliv og hvilke IT-virksomheder, der er de mest attraktive. Derudover handler den om brugen af AI på arbejdspladsen. Det tager 8-10 minutter at deltage, afhængig af besvarelsen kan tiden variere.</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Hvad er vigtigtst i dit arbejdsliv? - yihengldavid@gmail.com - Gmail</v>
+      </c>
+      <c r="N34" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
+      </c>
+      <c r="O34" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=deltage</v>
+      </c>
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
+      <c r="S34" t="str">
+        <v/>
+      </c>
+      <c r="T34" t="str">
+        <v/>
+      </c>
+      <c r="U34" t="str">
+        <v/>
+      </c>
+      <c r="V34" t="str">
+        <v/>
+      </c>
+      <c r="W34" t="str">
+        <v/>
+      </c>
+      <c r="X34" t="str">
+        <v/>
+      </c>
+      <c r="Y34" t="str">
+        <v/>
+      </c>
+      <c r="Z34" t="str">
+        <v/>
+      </c>
+      <c r="AA34" t="str">
+        <v/>
+      </c>
+      <c r="AB34" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB34"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "besvarelsen" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB34"/>
+  <dimension ref="A1:AB35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3134,9 +3134,95 @@
         <v/>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>244e9f09-9eb1-43d3-b89c-2f4d8ed0d52b</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C35" t="str">
+        <v>besvarelsen</v>
+      </c>
+      <c r="D35" t="str">
+        <v>besvarelse</v>
+      </c>
+      <c r="E35" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F35" t="str">
+        <v>en</v>
+      </c>
+      <c r="G35" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H35" t="str">
+        <v>[beˈsvɑˀɑlsə]</v>
+      </c>
+      <c r="I35" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004349_1.mp3</v>
+      </c>
+      <c r="J35" t="str">
+        <v>det at svare på et spørgsmål, en henvendelse, en forespørgsel el.lign.</v>
+      </c>
+      <c r="K35" t="str">
+        <v>The answer</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Undersøgelsen handler om, hvad der er vigtigt i dit arbejdsliv og hvilke IT-virksomheder, der er de mest attraktive. Derudover handler den om brugen af AI på arbejdspladsen. Det tager 8-10 minutter at deltage, afhængig af besvarelsen kan tiden variere.</v>
+      </c>
+      <c r="M35" t="str">
+        <v>Hvad er vigtigtst i dit arbejdsliv? - yihengldavid@gmail.com - Gmail</v>
+      </c>
+      <c r="N35" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
+      </c>
+      <c r="O35" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=besvarelsen</v>
+      </c>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R35" t="str">
+        <v/>
+      </c>
+      <c r="S35" t="str">
+        <v/>
+      </c>
+      <c r="T35" t="str">
+        <v/>
+      </c>
+      <c r="U35" t="str">
+        <v/>
+      </c>
+      <c r="V35" t="str">
+        <v/>
+      </c>
+      <c r="W35" t="str">
+        <v/>
+      </c>
+      <c r="X35" t="str">
+        <v/>
+      </c>
+      <c r="Y35" t="str">
+        <v/>
+      </c>
+      <c r="Z35" t="str">
+        <v/>
+      </c>
+      <c r="AA35" t="str">
+        <v/>
+      </c>
+      <c r="AB35" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB35"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Lodtrækningen" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB35"/>
+  <dimension ref="A1:AB36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3220,9 +3220,95 @@
         <v/>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>05e1e3ad-3bca-41f5-8e60-863c91b28803</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Lodtrækningen</v>
+      </c>
+      <c r="D36" t="str">
+        <v>lodtrækning</v>
+      </c>
+      <c r="E36" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F36" t="str">
+        <v>en</v>
+      </c>
+      <c r="G36" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v>https://static.ordnet.dk/mp3/11030/11030798_1.mp3</v>
+      </c>
+      <c r="J36" t="str">
+        <v>tildeling af fx gevinster, arbejdsopgaver eller modstandere i en sportsturnering ved tilfældig udvælgelse, ved udtrækning af mærkede eller nummererede sedler eller brikker el.lign. foretages fx i et lotteri, hvor der til hver lodseddel svarer et numm</v>
+      </c>
+      <c r="K36" t="str">
+        <v>The draw</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Lodtrækningen om ugentlige gavekort på 200 kr. og hovedpræmie på 10.000 kr.</v>
+      </c>
+      <c r="M36" t="str">
+        <v>Hvad er vigtigtst i dit arbejdsliv? - yihengldavid@gmail.com - Gmail</v>
+      </c>
+      <c r="N36" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
+      </c>
+      <c r="O36" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=Lodtr%C3%A6kningen</v>
+      </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R36" t="str">
+        <v/>
+      </c>
+      <c r="S36" t="str">
+        <v/>
+      </c>
+      <c r="T36" t="str">
+        <v/>
+      </c>
+      <c r="U36" t="str">
+        <v/>
+      </c>
+      <c r="V36" t="str">
+        <v/>
+      </c>
+      <c r="W36" t="str">
+        <v/>
+      </c>
+      <c r="X36" t="str">
+        <v/>
+      </c>
+      <c r="Y36" t="str">
+        <v/>
+      </c>
+      <c r="Z36" t="str">
+        <v/>
+      </c>
+      <c r="AA36" t="str">
+        <v/>
+      </c>
+      <c r="AB36" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB36"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "ugentlige" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB36"/>
+  <dimension ref="A1:AB37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3306,9 +3306,95 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>bd12ca48-9bef-4aca-b61e-a9c1461541d0</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C37" t="str">
+        <v>ugentlige</v>
+      </c>
+      <c r="D37" t="str">
+        <v>ugentlig</v>
+      </c>
+      <c r="E37" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H37" t="str">
+        <v>[ˈuːəndli]</v>
+      </c>
+      <c r="I37" t="str">
+        <v>https://static.ordnet.dk/mp3/12004/12004458_1.mp3</v>
+      </c>
+      <c r="J37" t="str">
+        <v>som finder sted, er til stede eller gøres hver uge</v>
+      </c>
+      <c r="K37" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Lodtrækningen om ugentlige gavekort på 200 kr. og hovedpræmie på 10.000 kr.</v>
+      </c>
+      <c r="M37" t="str">
+        <v>Hvad er vigtigtst i dit arbejdsliv? - yihengldavid@gmail.com - Gmail</v>
+      </c>
+      <c r="N37" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
+      </c>
+      <c r="O37" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=ugentlige</v>
+      </c>
+      <c r="P37" t="str">
+        <v/>
+      </c>
+      <c r="Q37" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R37" t="str">
+        <v/>
+      </c>
+      <c r="S37" t="str">
+        <v/>
+      </c>
+      <c r="T37" t="str">
+        <v/>
+      </c>
+      <c r="U37" t="str">
+        <v/>
+      </c>
+      <c r="V37" t="str">
+        <v/>
+      </c>
+      <c r="W37" t="str">
+        <v/>
+      </c>
+      <c r="X37" t="str">
+        <v/>
+      </c>
+      <c r="Y37" t="str">
+        <v/>
+      </c>
+      <c r="Z37" t="str">
+        <v/>
+      </c>
+      <c r="AA37" t="str">
+        <v/>
+      </c>
+      <c r="AB37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB37"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "vedrørende" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB37"/>
+  <dimension ref="A1:AB38"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3392,9 +3392,95 @@
         <v/>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>ee7ef30e-90ab-4172-8d3c-f42192b17545</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C38" t="str">
+        <v>vedrørende</v>
+      </c>
+      <c r="D38" t="str">
+        <v>vedrørende</v>
+      </c>
+      <c r="E38" t="str">
+        <v>præposition</v>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v>[-ˌʁɶˀʌnə]</v>
+      </c>
+      <c r="I38" t="str">
+        <v>https://static.ordnet.dk/mp3/12006/12006017_1.mp3</v>
+      </c>
+      <c r="J38" t="str">
+        <v>omhandlende, om; med tilknytning til</v>
+      </c>
+      <c r="K38" t="str">
+        <v>concerning</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Du har mulighed for at modtage information vedrørende din flyttesags forløb. Informationen sendes til din digitale postkasse. En tilhørende advisering via SMS om ny post i den digitale postkasse kan tilvælges.</v>
+      </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+      <c r="N38" t="str">
+        <v>https://notuseborger.scandihealth.net/EDS/eflyt/kontaktinfo.aspx</v>
+      </c>
+      <c r="O38" t="str">
+        <v>https://notuseborger.scandihealth.net/EDS/eflyt/kontaktinfo.aspx#:~:text=vedr%C3%B8rende</v>
+      </c>
+      <c r="P38" t="str">
+        <v/>
+      </c>
+      <c r="Q38" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R38" t="str">
+        <v/>
+      </c>
+      <c r="S38" t="str">
+        <v/>
+      </c>
+      <c r="T38" t="str">
+        <v/>
+      </c>
+      <c r="U38" t="str">
+        <v/>
+      </c>
+      <c r="V38" t="str">
+        <v/>
+      </c>
+      <c r="W38" t="str">
+        <v/>
+      </c>
+      <c r="X38" t="str">
+        <v/>
+      </c>
+      <c r="Y38" t="str">
+        <v/>
+      </c>
+      <c r="Z38" t="str">
+        <v/>
+      </c>
+      <c r="AA38" t="str">
+        <v/>
+      </c>
+      <c r="AB38" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB38"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Angive" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB38"/>
+  <dimension ref="A1:AB39"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3478,9 +3478,95 @@
         <v/>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>897bff27-e678-4acc-91bc-e6b7d2a95e09</v>
+      </c>
+      <c r="B39" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Angive</v>
+      </c>
+      <c r="D39" t="str">
+        <v>angive</v>
+      </c>
+      <c r="E39" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <v>-r, angav, -t</v>
+      </c>
+      <c r="H39" t="str">
+        <v>[ˈanˌgiˀ]</v>
+      </c>
+      <c r="I39" t="str">
+        <v>https://static.ordnet.dk/mp3/11001/11001769_1.mp3</v>
+      </c>
+      <c r="J39" t="str">
+        <v>oplyse eller meddele skriftligt eller mundtligt</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Indicate</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Angive årsagen til lægeskiftet, og hvornår det skal træde i kraft</v>
+      </c>
+      <c r="M39" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N39" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="O39" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=Angive</v>
+      </c>
+      <c r="P39" t="str">
+        <v/>
+      </c>
+      <c r="Q39" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R39" t="str">
+        <v/>
+      </c>
+      <c r="S39" t="str">
+        <v/>
+      </c>
+      <c r="T39" t="str">
+        <v/>
+      </c>
+      <c r="U39" t="str">
+        <v/>
+      </c>
+      <c r="V39" t="str">
+        <v/>
+      </c>
+      <c r="W39" t="str">
+        <v/>
+      </c>
+      <c r="X39" t="str">
+        <v/>
+      </c>
+      <c r="Y39" t="str">
+        <v/>
+      </c>
+      <c r="Z39" t="str">
+        <v/>
+      </c>
+      <c r="AA39" t="str">
+        <v/>
+      </c>
+      <c r="AB39" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB39"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "årsagen" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB39"/>
+  <dimension ref="A1:AB40"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3564,9 +3564,95 @@
         <v/>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>673c1a90-9c91-4f96-a37d-2642f01e292e</v>
+      </c>
+      <c r="B40" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C40" t="str">
+        <v>årsagen</v>
+      </c>
+      <c r="D40" t="str">
+        <v>årsag</v>
+      </c>
+      <c r="E40" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F40" t="str">
+        <v>en</v>
+      </c>
+      <c r="G40" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H40" t="str">
+        <v>[ˈɒːˌsæˀj]</v>
+      </c>
+      <c r="I40" t="str">
+        <v>https://static.ordnet.dk/mp3/12008/12008589_1.mp3</v>
+      </c>
+      <c r="J40" t="str">
+        <v>handling, begivenhed eller forhold som direkte bevirker, fremkalder eller resulterer i at noget forholder sig på en bestemt måde</v>
+      </c>
+      <c r="K40" t="str">
+        <v>The reason</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Angive årsagen til lægeskiftet, og hvornår det skal træde i kraft</v>
+      </c>
+      <c r="M40" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N40" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="O40" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=%C3%A5rsagen</v>
+      </c>
+      <c r="P40" t="str">
+        <v/>
+      </c>
+      <c r="Q40" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R40" t="str">
+        <v/>
+      </c>
+      <c r="S40" t="str">
+        <v/>
+      </c>
+      <c r="T40" t="str">
+        <v/>
+      </c>
+      <c r="U40" t="str">
+        <v/>
+      </c>
+      <c r="V40" t="str">
+        <v/>
+      </c>
+      <c r="W40" t="str">
+        <v/>
+      </c>
+      <c r="X40" t="str">
+        <v/>
+      </c>
+      <c r="Y40" t="str">
+        <v/>
+      </c>
+      <c r="Z40" t="str">
+        <v/>
+      </c>
+      <c r="AA40" t="str">
+        <v/>
+      </c>
+      <c r="AB40" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB40"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "træde" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB40"/>
+  <dimension ref="A1:AB41"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3650,9 +3650,95 @@
         <v/>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>6504e35c-6d7a-4741-a2ba-072467ee7383</v>
+      </c>
+      <c r="B41" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C41" t="str">
+        <v>træde</v>
+      </c>
+      <c r="D41" t="str">
+        <v>træde</v>
+      </c>
+      <c r="E41" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v>-r, trådte, trådt</v>
+      </c>
+      <c r="H41" t="str">
+        <v>[ˈtʁεːðə]</v>
+      </c>
+      <c r="I41" t="str">
+        <v>https://static.ordnet.dk/mp3/12002/12002632_1.mp3</v>
+      </c>
+      <c r="J41" t="str">
+        <v>tage et eller flere skridt til et sted (hvor man derefter standser)</v>
+      </c>
+      <c r="K41" t="str">
+        <v>step</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Angive årsagen til lægeskiftet, og hvornår det skal træde i kraft</v>
+      </c>
+      <c r="M41" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N41" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="O41" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=tr%C3%A6de</v>
+      </c>
+      <c r="P41" t="str">
+        <v/>
+      </c>
+      <c r="Q41" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R41" t="str">
+        <v/>
+      </c>
+      <c r="S41" t="str">
+        <v/>
+      </c>
+      <c r="T41" t="str">
+        <v/>
+      </c>
+      <c r="U41" t="str">
+        <v/>
+      </c>
+      <c r="V41" t="str">
+        <v/>
+      </c>
+      <c r="W41" t="str">
+        <v/>
+      </c>
+      <c r="X41" t="str">
+        <v/>
+      </c>
+      <c r="Y41" t="str">
+        <v/>
+      </c>
+      <c r="Z41" t="str">
+        <v/>
+      </c>
+      <c r="AA41" t="str">
+        <v/>
+      </c>
+      <c r="AB41" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB41"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "kraft" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB41"/>
+  <dimension ref="A1:AB42"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3736,9 +3736,95 @@
         <v/>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>ad92ed40-c154-443a-b59d-8be143477ce4</v>
+      </c>
+      <c r="B42" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C42" t="str">
+        <v>kraft</v>
+      </c>
+      <c r="D42" t="str">
+        <v>kraft</v>
+      </c>
+      <c r="E42" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F42" t="str">
+        <v>en</v>
+      </c>
+      <c r="G42" t="str">
+        <v>-en, kræfter, kræfterne</v>
+      </c>
+      <c r="H42" t="str">
+        <v>[ˈkʁɑfd]</v>
+      </c>
+      <c r="I42" t="str">
+        <v>https://static.ordnet.dk/mp3/11027/11027868_1.mp3</v>
+      </c>
+      <c r="J42" t="str">
+        <v>fysisk fænomen der viser sig som evnen til at forandre et legemes bevægelse eller tilstand</v>
+      </c>
+      <c r="K42" t="str">
+        <v>force</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Angive årsagen til lægeskiftet, og hvornår det skal træde i kraft</v>
+      </c>
+      <c r="M42" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N42" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="O42" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=kraft</v>
+      </c>
+      <c r="P42" t="str">
+        <v/>
+      </c>
+      <c r="Q42" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R42" t="str">
+        <v/>
+      </c>
+      <c r="S42" t="str">
+        <v/>
+      </c>
+      <c r="T42" t="str">
+        <v/>
+      </c>
+      <c r="U42" t="str">
+        <v/>
+      </c>
+      <c r="V42" t="str">
+        <v/>
+      </c>
+      <c r="W42" t="str">
+        <v/>
+      </c>
+      <c r="X42" t="str">
+        <v/>
+      </c>
+      <c r="Y42" t="str">
+        <v/>
+      </c>
+      <c r="Z42" t="str">
+        <v/>
+      </c>
+      <c r="AA42" t="str">
+        <v/>
+      </c>
+      <c r="AB42" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB42"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "træde i kraft" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB42"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3831,30 +3831,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4129,9 +4129,77 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>75396d64-26c5-41b5-b4ef-8aa33ef958b3</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C5" t="str">
+        <v>træde i kraft</v>
+      </c>
+      <c r="D5" t="str">
+        <v>træde=step · i=in · kraft=force</v>
+      </c>
+      <c r="E5" t="str">
+        <v>take effect</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Angive årsagen til lægeskiftet, og hvornår det skal træde i kraft</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="H5" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=tr%C3%A6de%20i%20kraft</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "kræves" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB42"/>
+  <dimension ref="A1:AB43"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3822,9 +3822,95 @@
         <v/>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>2ed1e140-78a2-4201-8653-c6cb8b38e202</v>
+      </c>
+      <c r="B43" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C43" t="str">
+        <v>kræves</v>
+      </c>
+      <c r="D43" t="str">
+        <v>kræve</v>
+      </c>
+      <c r="E43" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H43" t="str">
+        <v>[ˈkʁεːvə]</v>
+      </c>
+      <c r="I43" t="str">
+        <v>https://static.ordnet.dk/mp3/11028/11028389_1.mp3</v>
+      </c>
+      <c r="J43" t="str">
+        <v>stille krav om at noget bestemt gennemføres, sættes i værk, bevilges el.lign.; forlange at et ønske opfyldes</v>
+      </c>
+      <c r="K43" t="str">
+        <v>required</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Betale for lægeskift vha. betalingskort, hvis dette kræves</v>
+      </c>
+      <c r="M43" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N43" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="O43" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=kr%C3%A6ves</v>
+      </c>
+      <c r="P43" t="str">
+        <v/>
+      </c>
+      <c r="Q43" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R43" t="str">
+        <v/>
+      </c>
+      <c r="S43" t="str">
+        <v/>
+      </c>
+      <c r="T43" t="str">
+        <v/>
+      </c>
+      <c r="U43" t="str">
+        <v/>
+      </c>
+      <c r="V43" t="str">
+        <v/>
+      </c>
+      <c r="W43" t="str">
+        <v/>
+      </c>
+      <c r="X43" t="str">
+        <v/>
+      </c>
+      <c r="Y43" t="str">
+        <v/>
+      </c>
+      <c r="Z43" t="str">
+        <v/>
+      </c>
+      <c r="AA43" t="str">
+        <v/>
+      </c>
+      <c r="AB43" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB43"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3833,28 +3919,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V5"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "nuværende" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB43"/>
+  <dimension ref="A1:AB44"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3908,9 +3908,95 @@
         <v/>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>f4880534-2f86-4124-bd54-fbd3f1eee632</v>
+      </c>
+      <c r="B44" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C44" t="str">
+        <v>nuværende</v>
+      </c>
+      <c r="D44" t="str">
+        <v>nuværende</v>
+      </c>
+      <c r="E44" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F44" t="str">
+        <v>en</v>
+      </c>
+      <c r="G44" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
+      <c r="I44" t="str">
+        <v/>
+      </c>
+      <c r="J44" t="str">
+        <v>sammensat af nuvæ + rende</v>
+      </c>
+      <c r="K44" t="str">
+        <v>present</v>
+      </c>
+      <c r="L44" t="str">
+        <v>Det er gratis at skifte læge, hvis din nuværende læge lukker sin praksis eller hvis du skifter læge i forbindelse med en flytning.</v>
+      </c>
+      <c r="M44" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N44" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="O44" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=nuv%C3%A6rende</v>
+      </c>
+      <c r="P44" t="str">
+        <v/>
+      </c>
+      <c r="Q44" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R44" t="str">
+        <v/>
+      </c>
+      <c r="S44" t="str">
+        <v/>
+      </c>
+      <c r="T44" t="str">
+        <v/>
+      </c>
+      <c r="U44" t="str">
+        <v/>
+      </c>
+      <c r="V44" t="str">
+        <v/>
+      </c>
+      <c r="W44" t="str">
+        <v/>
+      </c>
+      <c r="X44" t="str">
+        <v/>
+      </c>
+      <c r="Y44" t="str">
+        <v/>
+      </c>
+      <c r="Z44" t="str">
+        <v/>
+      </c>
+      <c r="AA44" t="str">
+        <v/>
+      </c>
+      <c r="AB44" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB44"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "gebyrfrit" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB44"/>
+  <dimension ref="A1:AB45"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3994,9 +3994,95 @@
         <v/>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>197a7301-54e7-48bb-a9df-c2bac234a291</v>
+      </c>
+      <c r="B45" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C45" t="str">
+        <v>gebyrfrit</v>
+      </c>
+      <c r="D45" t="str">
+        <v>gebyrfri</v>
+      </c>
+      <c r="E45" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <v>-t, - eller -e Se bøjning i skema</v>
+      </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
+      <c r="I45" t="str">
+        <v>https://static.ordnet.dk/mp3/53201/53201522_1.mp3</v>
+      </c>
+      <c r="J45" t="str">
+        <v>som man ikke betaler gebyr for</v>
+      </c>
+      <c r="K45" t="str">
+        <v>fee-free</v>
+      </c>
+      <c r="L45" t="str">
+        <v>Hvis du vælger at beholde din nuværende læge ved din flytning, kan du ikke senere skifte læge gebyrfrit.</v>
+      </c>
+      <c r="M45" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N45" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="O45" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=gebyrfrit</v>
+      </c>
+      <c r="P45" t="str">
+        <v/>
+      </c>
+      <c r="Q45" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R45" t="str">
+        <v/>
+      </c>
+      <c r="S45" t="str">
+        <v/>
+      </c>
+      <c r="T45" t="str">
+        <v/>
+      </c>
+      <c r="U45" t="str">
+        <v/>
+      </c>
+      <c r="V45" t="str">
+        <v/>
+      </c>
+      <c r="W45" t="str">
+        <v/>
+      </c>
+      <c r="X45" t="str">
+        <v/>
+      </c>
+      <c r="Y45" t="str">
+        <v/>
+      </c>
+      <c r="Z45" t="str">
+        <v/>
+      </c>
+      <c r="AA45" t="str">
+        <v/>
+      </c>
+      <c r="AB45" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB45"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "angivne" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB45"/>
+  <dimension ref="A1:AB46"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4080,9 +4080,95 @@
         <v/>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>124879d2-1f9b-4f7f-81bf-3fc738143f1d</v>
+      </c>
+      <c r="B46" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C46" t="str">
+        <v>angivne</v>
+      </c>
+      <c r="D46" t="str">
+        <v>angive</v>
+      </c>
+      <c r="E46" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46" t="str">
+        <v>-r, angav, -t</v>
+      </c>
+      <c r="H46" t="str">
+        <v>[ˈanˌgiˀ]</v>
+      </c>
+      <c r="I46" t="str">
+        <v>https://static.ordnet.dk/mp3/11001/11001769_1.mp3</v>
+      </c>
+      <c r="J46" t="str">
+        <v>oplyse eller meddele skriftligt eller mundtligt</v>
+      </c>
+      <c r="K46" t="str">
+        <v>indicated</v>
+      </c>
+      <c r="L46" t="str">
+        <v>Hvis lægeskiftet sker i forbindelse med lukning eller ændringer af din nuværende læges praksis, skal lægeskiftet ske inden for den angivne periode, der fremgår at det brev du har modtaget fra regionen.</v>
+      </c>
+      <c r="M46" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N46" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="O46" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=angivne</v>
+      </c>
+      <c r="P46" t="str">
+        <v/>
+      </c>
+      <c r="Q46" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R46" t="str">
+        <v/>
+      </c>
+      <c r="S46" t="str">
+        <v/>
+      </c>
+      <c r="T46" t="str">
+        <v/>
+      </c>
+      <c r="U46" t="str">
+        <v/>
+      </c>
+      <c r="V46" t="str">
+        <v/>
+      </c>
+      <c r="W46" t="str">
+        <v/>
+      </c>
+      <c r="X46" t="str">
+        <v/>
+      </c>
+      <c r="Y46" t="str">
+        <v/>
+      </c>
+      <c r="Z46" t="str">
+        <v/>
+      </c>
+      <c r="AA46" t="str">
+        <v/>
+      </c>
+      <c r="AB46" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB46"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "trin" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB46"/>
+  <dimension ref="A1:AB47"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4166,9 +4166,95 @@
         <v/>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>1f470a0e-1db4-4dbd-b080-08f7633f9d04</v>
+      </c>
+      <c r="B47" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C47" t="str">
+        <v>trin</v>
+      </c>
+      <c r="D47" t="str">
+        <v>trin</v>
+      </c>
+      <c r="E47" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F47" t="str">
+        <v>et</v>
+      </c>
+      <c r="G47" t="str">
+        <v>-net eller -et, -, -nene eller -ene</v>
+      </c>
+      <c r="H47" t="str">
+        <v>[ˈtʁin]</v>
+      </c>
+      <c r="I47" t="str">
+        <v>https://static.ordnet.dk/mp3/12002/12002377_1.mp3</v>
+      </c>
+      <c r="J47" t="str">
+        <v>(smal) flade til at træde op på undervejs til et højere niveau; ofte placeret over en tilsvarende flade, fx som del af en trappe eller en stige</v>
+      </c>
+      <c r="K47" t="str">
+        <v>step</v>
+      </c>
+      <c r="L47" t="str">
+        <v>Hvis lægeskiftet sker i forbindelse med flytning, vil lægevalget først blive godkendt når flytningen er godkendt. Lægevalg i forbindelse med flytning, er kun gebyrfrit så længe flytningen ikke er godkendt. Hvis din tilflytningsadresse ligger i en anden kommune, vil du i næste trin blive bedt om at skifte kommune.</v>
+      </c>
+      <c r="M47" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N47" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="O47" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=trin</v>
+      </c>
+      <c r="P47" t="str">
+        <v/>
+      </c>
+      <c r="Q47" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R47" t="str">
+        <v/>
+      </c>
+      <c r="S47" t="str">
+        <v/>
+      </c>
+      <c r="T47" t="str">
+        <v/>
+      </c>
+      <c r="U47" t="str">
+        <v/>
+      </c>
+      <c r="V47" t="str">
+        <v/>
+      </c>
+      <c r="W47" t="str">
+        <v/>
+      </c>
+      <c r="X47" t="str">
+        <v/>
+      </c>
+      <c r="Y47" t="str">
+        <v/>
+      </c>
+      <c r="Z47" t="str">
+        <v/>
+      </c>
+      <c r="AA47" t="str">
+        <v/>
+      </c>
+      <c r="AB47" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB47"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "blive bedt om" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB47"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4261,30 +4261,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V6"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4627,9 +4627,77 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>a49b080c-576d-4263-b98a-11b39922fd8c</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C6" t="str">
+        <v>blive bedt om</v>
+      </c>
+      <c r="D6" t="str">
+        <v>blive=be · bedt=prayed · om=on</v>
+      </c>
+      <c r="E6" t="str">
+        <v>be asked for</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Hvis lægeskiftet sker i forbindelse med flytning, vil lægevalget først blive godkendt når flytningen er godkendt. Lægevalg i forbindelse med flytning, er kun gebyrfrit så længe flytningen ikke er godkendt. Hvis din tilflytningsadresse ligger i en anden kommune, vil du i næste trin blive bedt om at skifte kommune.</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="H6" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=blive%20bedt%20om</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bedt" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB47"/>
+  <dimension ref="A1:AB48"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4252,9 +4252,95 @@
         <v/>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>39478c50-787c-4139-8af5-3b86301a5a23</v>
+      </c>
+      <c r="B48" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C48" t="str">
+        <v>bedt</v>
+      </c>
+      <c r="D48" t="str">
+        <v>bede</v>
+      </c>
+      <c r="E48" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v>-r, bad (eller uofficiel form: bedte), bedt Se bøjning i skema</v>
+      </c>
+      <c r="H48" t="str">
+        <v>[ˈbeˀ]</v>
+      </c>
+      <c r="I48" t="str">
+        <v>https://static.ordnet.dk/mp3/11003/11003719_1.mp3</v>
+      </c>
+      <c r="J48" t="str">
+        <v>søge at opnå noget hos en anden person</v>
+      </c>
+      <c r="K48" t="str">
+        <v>prayed</v>
+      </c>
+      <c r="L48" t="str">
+        <v>Hvis lægeskiftet sker i forbindelse med flytning, vil lægevalget først blive godkendt når flytningen er godkendt. Lægevalg i forbindelse med flytning, er kun gebyrfrit så længe flytningen ikke er godkendt. Hvis din tilflytningsadresse ligger i en anden kommune, vil du i næste trin blive bedt om at skifte kommune.</v>
+      </c>
+      <c r="M48" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N48" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461</v>
+      </c>
+      <c r="O48" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0461#:~:text=bedt</v>
+      </c>
+      <c r="P48" t="str">
+        <v/>
+      </c>
+      <c r="Q48" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R48" t="str">
+        <v/>
+      </c>
+      <c r="S48" t="str">
+        <v/>
+      </c>
+      <c r="T48" t="str">
+        <v/>
+      </c>
+      <c r="U48" t="str">
+        <v/>
+      </c>
+      <c r="V48" t="str">
+        <v/>
+      </c>
+      <c r="W48" t="str">
+        <v/>
+      </c>
+      <c r="X48" t="str">
+        <v/>
+      </c>
+      <c r="Y48" t="str">
+        <v/>
+      </c>
+      <c r="Z48" t="str">
+        <v/>
+      </c>
+      <c r="AA48" t="str">
+        <v/>
+      </c>
+      <c r="AB48" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB48"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4263,28 +4349,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V6"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "ikrafttrædelse" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB48"/>
+  <dimension ref="A1:AB49"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4338,9 +4338,95 @@
         <v/>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>3e25514e-debb-4b69-82f3-1b51132f64b1</v>
+      </c>
+      <c r="B49" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C49" t="str">
+        <v>ikrafttrædelse</v>
+      </c>
+      <c r="D49" t="str">
+        <v>ikrafttrædelse</v>
+      </c>
+      <c r="E49" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F49" t="str">
+        <v>en</v>
+      </c>
+      <c r="G49" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H49" t="str">
+        <v>[iˈkʁɑfdˌtʁεˀðəlsə]</v>
+      </c>
+      <c r="I49" t="str">
+        <v>https://static.ordnet.dk/mp3/11022/11022905_1.mp3</v>
+      </c>
+      <c r="J49" t="str">
+        <v>= ikrafttræden</v>
+      </c>
+      <c r="K49" t="str">
+        <v>Entry into force</v>
+      </c>
+      <c r="L49" t="str">
+        <v>Dato for ikrafttrædelse</v>
+      </c>
+      <c r="M49" t="str">
+        <v>Sygesikring</v>
+      </c>
+      <c r="N49" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0540&amp;isDueToRelocation=false</v>
+      </c>
+      <c r="O49" t="str">
+        <v>https://self-service-prod.prod.gultsundhedskort.dk/laegevalg?kommuneid=0540&amp;isDueToRelocation=false#:~:text=ikrafttr%C3%A6delse</v>
+      </c>
+      <c r="P49" t="str">
+        <v/>
+      </c>
+      <c r="Q49" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R49" t="str">
+        <v/>
+      </c>
+      <c r="S49" t="str">
+        <v/>
+      </c>
+      <c r="T49" t="str">
+        <v/>
+      </c>
+      <c r="U49" t="str">
+        <v/>
+      </c>
+      <c r="V49" t="str">
+        <v/>
+      </c>
+      <c r="W49" t="str">
+        <v/>
+      </c>
+      <c r="X49" t="str">
+        <v/>
+      </c>
+      <c r="Y49" t="str">
+        <v/>
+      </c>
+      <c r="Z49" t="str">
+        <v/>
+      </c>
+      <c r="AA49" t="str">
+        <v/>
+      </c>
+      <c r="AB49" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB49"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>